<commit_message>
Update Organization_Template_Alternate.xlsx: blank row before headers, asterisk-marked required columns, freeze panes
Structural edits made directly in the workbook: a blank row now
precedes the header row on every sheet except "How to use this
workbook" and "Main Org record"; required columns are now marked with
a trailing red "*" in the header text instead of a colored cell; and
every sheet now freezes the header row(s) plus the ORG CODE column
(matching the Interfaces tab's existing behavior) so both stay in view
while scrolling. Also renamed "ORG TYPE" to "ORG TYPE (Choose one or
create your own)" and "EXP ACTIVATION INTERVAL" to "EXPECTED
ACTIVATION INTERVAL", and added a LANGUAGE column to Emails.

The code changes needed to keep AlternateTemplateFlattener.php working
with all of this were already committed separately.
</commit_message>
<xml_diff>
--- a/Organization_Template_Alternate.xlsx
+++ b/Organization_Template_Alternate.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-37452" yWindow="10548" windowWidth="21744" windowHeight="11844" tabRatio="731" firstSheet="8" activeTab="8" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1650" yWindow="1455" windowWidth="25050" windowHeight="13140" tabRatio="731" firstSheet="1" activeTab="11" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="How to use this workbook" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,14 +20,14 @@
     <sheet name="External note" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,22 +90,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Aptos"/>
-      <charset val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
-      <charset val="1"/>
-      <color rgb="FF242424"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Source Sans Pro"/>
-      <i val="1"/>
-      <color theme="0" tint="-0.499984740745262"/>
-      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -164,7 +161,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -177,39 +174,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
@@ -218,16 +192,30 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -609,7 +597,7 @@
   <dimension ref="B2:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.140625" customWidth="1" min="2" max="2"/>
+    <col width="12.140625" customWidth="1" style="24" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -641,14 +629,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Go to Main Org record sheet</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Please note that coloured columns are mandatory.</t>
         </is>
@@ -689,86 +677,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14.42578125" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="14"/>
+    <col width="14.42578125" customWidth="1" style="24" min="1" max="1"/>
+    <col width="15" customWidth="1" style="24" min="2" max="10"/>
+    <col width="15" customWidth="1" style="12" min="11" max="11"/>
+    <col width="15" customWidth="1" style="24" min="12" max="13"/>
+    <col width="15" customWidth="1" style="12" min="14" max="14"/>
+    <col width="11.42578125" bestFit="1" customWidth="1" style="24" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="27" t="inlineStr">
+    <row r="1" ht="60" customHeight="1" s="24">
+      <c r="C1" s="19" t="inlineStr">
+        <is>
+          <t>Pipe delimited (|) list of currencies permitted</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1" s="24">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>PAYMENT METHOD</t>
         </is>
       </c>
-      <c r="C1" s="27" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>CURRENCIES</t>
         </is>
       </c>
-      <c r="D1" s="27" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>CLAIMING INTERVAL</t>
         </is>
       </c>
-      <c r="E1" s="27" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>DISCOUNT %</t>
         </is>
       </c>
-      <c r="F1" s="27" t="inlineStr">
-        <is>
-          <t>EXP ACTIVATION INTERVAL</t>
-        </is>
-      </c>
-      <c r="G1" s="27" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>EXPECTED ACTIVATION INTERVAL</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>EXP INVOICE INTERVAL</t>
         </is>
       </c>
-      <c r="H1" s="27" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>EXP RECEIPT INTERVAL</t>
         </is>
       </c>
-      <c r="I1" s="27" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>RENEWAL ACTIVATION INTERVAL</t>
         </is>
       </c>
-      <c r="J1" s="27" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>SUBSCRIPTION INTERVAL</t>
         </is>
       </c>
-      <c r="K1" s="27" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>EXPORT TO ACCOUNTING (Y/)</t>
         </is>
       </c>
-      <c r="L1" s="27" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>TAX ID</t>
         </is>
       </c>
-      <c r="M1" s="27" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>TAX %</t>
         </is>
       </c>
-      <c r="N1" s="27" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>LIABLE FOR VAT (Y/N)</t>
         </is>
       </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Do not edit:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="K3:K1048576" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>$AA$2:$AA$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="N3:N1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -779,127 +798,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A2:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.28515625" customWidth="1" style="20" min="1" max="1"/>
-    <col width="22.140625" customWidth="1" min="2" max="2"/>
-    <col width="20.85546875" customWidth="1" min="3" max="3"/>
-    <col width="36.5703125" customWidth="1" min="4" max="4"/>
-    <col width="24.5703125" customWidth="1" min="5" max="6"/>
-    <col width="25.85546875" customWidth="1" min="7" max="7"/>
-    <col width="18.85546875" customWidth="1" style="15" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13.28515625" customWidth="1" style="23" min="1" max="1"/>
+    <col width="22.140625" customWidth="1" style="24" min="2" max="2"/>
+    <col width="20.85546875" customWidth="1" style="24" min="3" max="3"/>
+    <col width="36.5703125" customWidth="1" style="24" min="4" max="4"/>
+    <col width="24.5703125" customWidth="1" style="24" min="5" max="6"/>
+    <col width="25.85546875" customWidth="1" style="24" min="7" max="7"/>
+    <col width="18.85546875" customWidth="1" style="8" min="8" max="8"/>
+    <col width="20" customWidth="1" style="24" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="24">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="22" t="inlineStr">
-        <is>
-          <t>ACCOUNT NAME</t>
-        </is>
-      </c>
-      <c r="C1" s="30" t="inlineStr">
-        <is>
-          <t>ACCOUNT NUMBER</t>
-        </is>
-      </c>
-      <c r="D1" s="23" t="inlineStr">
+    <row r="2" customFormat="1" s="10">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>ACCOUNT NAME*</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>ACCOUNT NUMBER*</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>ACCOUNTING CODE</t>
         </is>
       </c>
-      <c r="F1" s="23" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>PAYMENT METHOD</t>
         </is>
       </c>
-      <c r="G1" s="30" t="inlineStr">
-        <is>
-          <t>ACCOUNT STATUS</t>
-        </is>
-      </c>
-      <c r="H1" s="26" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
+        <is>
+          <t>ACCOUNT STATUS*</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>LIBRARY EDI CODE</t>
         </is>
       </c>
-      <c r="I1" s="23" t="inlineStr">
+      <c r="I2" s="22" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>EBSCO eBooks</t>
-        </is>
-      </c>
-      <c r="C2" s="25" t="n">
-        <v>12345</v>
-      </c>
-      <c r="D2" s="18" t="inlineStr">
-        <is>
-          <t>ebooks purchased from EBSCO</t>
-        </is>
-      </c>
-      <c r="E2" s="18" t="n"/>
-      <c r="F2" s="18" t="n"/>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H2" s="25" t="n">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>EBSCO databases</t>
-        </is>
-      </c>
-      <c r="C3" s="25" t="n">
-        <v>12346</v>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>databases purchased from EBSCO</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H3" s="25" t="n">
-        <v>456</v>
-      </c>
-    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G3:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Active,Inactive,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -910,32 +874,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A2:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.57" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="10.5703125" customWidth="1" style="24" min="1" max="1"/>
+    <col width="15" customWidth="1" style="24" min="2" max="2"/>
+    <col width="30" customWidth="1" style="24" min="3" max="3"/>
+    <col width="50" customWidth="1" style="24" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="31" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="31" t="inlineStr">
-        <is>
-          <t>NOTE TYPE</t>
-        </is>
-      </c>
-      <c r="C1" s="31" t="inlineStr">
-        <is>
-          <t>NOTE TITLE</t>
-        </is>
-      </c>
-      <c r="D1" s="28" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="24">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>NOTE TYPE*</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>NOTE TITLE*</t>
+        </is>
+      </c>
+      <c r="D2" s="25" t="inlineStr">
         <is>
           <t>CONTENTS</t>
         </is>
@@ -956,40 +920,40 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.42578125" customWidth="1" style="8" min="1" max="1"/>
-    <col width="25.42578125" customWidth="1" style="8" min="2" max="2"/>
-    <col width="11.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="16.140625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="35" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="11.42578125" customWidth="1" style="24" min="1" max="1"/>
+    <col width="25.42578125" customWidth="1" style="24" min="2" max="2"/>
+    <col width="16.140625" bestFit="1" customWidth="1" style="24" min="3" max="3"/>
+    <col width="36" bestFit="1" customWidth="1" style="24" min="4" max="4"/>
+    <col width="35" bestFit="1" customWidth="1" style="24" min="5" max="5"/>
+    <col width="40" bestFit="1" customWidth="1" style="24" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="B1" s="12" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1" s="24">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>NOTE: Unlike the original Organization_Template.xlsx, this sheet holds only the fields that can't repeat. Every address, phone number, email, URL, and alternative name for this organization - including the first one - belongs on the Addresses/Phones/Emails/URLs/Alt names sheet instead.</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18.75" customHeight="1">
-      <c r="B2" s="12" t="n"/>
+    <row r="2" ht="18.75" customHeight="1" s="24">
+      <c r="B2" s="14" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Coloured columns are mandatory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>ORG NAME</t>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Columns marked with * are mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" s="24">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>ORG NAME*</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -997,9 +961,9 @@
           <t>Vendor (Yes/No)</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>ORG status (Active/Inactive/Pending)</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ORG status (Active/Inactive/Pending)*</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1007,35 +971,30 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="F5" s="28" t="inlineStr">
-        <is>
-          <t>ORG TYPE</t>
+      <c r="F5" s="25" t="inlineStr">
+        <is>
+          <t>ORG TYPE (Choose one or create your own)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>EBSCO Information Services</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="5" t="n"/>
-      <c r="D6" s="10" t="n"/>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1"/>
+    <row r="7" ht="15.75" customHeight="1" s="24"/>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="C6:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
     <dataValidation sqref="D6:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Active, Inactive, Pending"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Access provider,Auction house,Book trade,Consortium,Content provider,Logistics,Material supplier,Membership organization,Private person,Publisher"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1049,26 +1008,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A2:C2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="7.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="15.42578125" customWidth="1" min="1" max="1"/>
-    <col width="11.42578125" customWidth="1" style="8" min="2" max="2"/>
-    <col width="13.28515625" customWidth="1" min="3" max="3"/>
+    <col width="15.42578125" customWidth="1" style="24" min="1" max="1"/>
+    <col width="12.7109375" customWidth="1" style="24" min="2" max="2"/>
+    <col width="13.28515625" customWidth="1" style="24" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>ALT NAME</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="24">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ALT NAME*</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -1085,66 +1044,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A2:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20.28515625" customWidth="1" min="1" max="1"/>
-    <col width="13.28515625" customWidth="1" min="6" max="6"/>
-    <col width="10.5703125" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20.28515625" customWidth="1" style="24" min="1" max="1"/>
+    <col width="45.7109375" customWidth="1" style="24" min="2" max="3"/>
+    <col width="13" customWidth="1" style="24" min="5" max="5"/>
+    <col width="13.28515625" customWidth="1" style="24" min="6" max="6"/>
+    <col width="14.5703125" customWidth="1" style="24" min="7" max="7"/>
+    <col width="19.42578125" customWidth="1" style="24" min="8" max="8"/>
+    <col width="14" customWidth="1" style="24" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="24">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ADDR1 </t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>ADDR2</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CITY</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>REGION</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>POSTAL CODE</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>COUNTRY</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="I1" s="28" t="inlineStr">
+      <c r="I2" s="25" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="I3:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes, No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1157,85 +1122,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A2:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16.7109375" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" style="8" min="2" max="2"/>
-    <col width="10.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16.7109375" customWidth="1" style="24" min="1" max="1"/>
+    <col width="15" customWidth="1" style="24" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" style="24" min="4" max="4"/>
+    <col width="14" customWidth="1" style="24" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>PHONE</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="24">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PHONE*</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="25" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>800-653-2726</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>800-633-4604</t>
-        </is>
-      </c>
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
       <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="C3:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Office, Mobile, Fax, Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes, No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D3:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1248,71 +1190,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A2:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18.140625" customWidth="1" min="1" max="1"/>
-    <col width="27.140625" customWidth="1" style="8" min="2" max="2"/>
-    <col width="27.140625" customWidth="1" min="3" max="3"/>
-    <col width="10.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18.140625" customWidth="1" style="24" min="1" max="1"/>
+    <col width="27.140625" customWidth="1" style="24" min="2" max="3"/>
+    <col width="11.140625" bestFit="1" customWidth="1" style="24" min="4" max="4"/>
+    <col width="14" customWidth="1" style="24" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>EMAIL</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="24">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>EMAIL*</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>LANGUAGE</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="F2" s="25" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>customerservice@ebsco.com</t>
-        </is>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>sales@ebsco.com</t>
-        </is>
-      </c>
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="E3:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes, No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D3:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1325,52 +1258,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A2:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18.140625" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18.140625" customWidth="1" style="24" min="1" max="1"/>
+    <col width="40" customWidth="1" style="24" min="2" max="2"/>
+    <col width="30" customWidth="1" style="24" min="3" max="4"/>
+    <col width="14" customWidth="1" style="24" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="31" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="31" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="C1" s="28" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>URL*</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
+      <c r="D2" s="25" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="25" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-      <c r="F1" s="28" t="inlineStr">
+      <c r="F2" s="25" t="inlineStr">
         <is>
           <t>IS PRIMARY</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="E4:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes, No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E3" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1383,129 +1318,87 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A2:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="20.25" customHeight="1"/>
   <cols>
-    <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="11.140625" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
-    <col width="11.7109375" bestFit="1" customWidth="1" style="8" min="3" max="3"/>
-    <col width="6.28515625" customWidth="1" min="4" max="4"/>
-    <col width="7.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="23.28515625" customWidth="1" style="8" min="6" max="6"/>
-    <col width="14.42578125" customWidth="1" style="8" min="7" max="7"/>
-    <col width="18.28515625" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="24" min="1" max="1"/>
+    <col width="12.140625" bestFit="1" customWidth="1" style="24" min="2" max="2"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" style="24" min="3" max="3"/>
+    <col width="12.42578125" customWidth="1" style="24" min="4" max="4"/>
+    <col width="24.85546875" customWidth="1" style="24" min="5" max="5"/>
+    <col width="23.28515625" customWidth="1" style="24" min="6" max="6"/>
+    <col width="14.42578125" customWidth="1" style="24" min="7" max="7"/>
+    <col width="18.28515625" customWidth="1" style="24" min="8" max="8"/>
+    <col width="13" customWidth="1" style="24" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customFormat="1" customHeight="1" s="3">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>LAST NAME</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>FIRST NAME</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+    <row r="2" ht="20.25" customFormat="1" customHeight="1" s="3">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>LAST NAME*</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>FIRST NAME*</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="E1" s="32" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="F1" s="32" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">PHONE </t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>CATEGORIES</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>Novak</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>jnovak@ebsco.com</t>
-        </is>
-      </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>555-555-5555</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Accounts receivable</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Rossi</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Mario</t>
-        </is>
-      </c>
+      <c r="J2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="20.25" customHeight="1" s="24">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>mrossi@ebsco.com</t>
-        </is>
-      </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>555-555-5555</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Customer service</t>
-        </is>
-      </c>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="20.25" customHeight="1" s="24">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H3:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1516,119 +1409,97 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="14.42578125" customWidth="1" style="8" min="2" max="2"/>
-    <col width="11.85546875" customWidth="1" min="3" max="3"/>
-    <col width="35.7109375" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="6"/>
-    <col width="13.28515625" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="13.140625" customWidth="1" min="8" max="8"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" style="24" min="1" max="1"/>
+    <col width="14.42578125" customWidth="1" style="24" min="2" max="2"/>
+    <col width="11.85546875" customWidth="1" style="24" min="3" max="3"/>
+    <col width="35.7109375" customWidth="1" style="24" min="4" max="4"/>
+    <col width="18" customWidth="1" style="24" min="5" max="6"/>
+    <col width="16.140625" customWidth="1" style="24" min="7" max="7"/>
+    <col width="13.140625" customWidth="1" style="24" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>ORG CODE</t>
-        </is>
-      </c>
-      <c r="B1" s="32" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="24">
+      <c r="F1" s="19" t="inlineStr">
+        <is>
+          <t>If a username is present, a password must be set as well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="24">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORG CODE*</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E2" s="25" t="inlineStr">
         <is>
           <t>DELIVERY METHOD</t>
         </is>
       </c>
-      <c r="F1" s="31" t="inlineStr">
+      <c r="F2" s="25" t="inlineStr">
         <is>
           <t>USERNAME</t>
         </is>
       </c>
-      <c r="G1" s="31" t="inlineStr">
+      <c r="G2" s="25" t="inlineStr">
         <is>
           <t>PASSWORD</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>EBSCO Admin</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>https://eadmin.ebscohost.com/eadmin</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>myuser</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>mypass</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="n"/>
-    </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>E.g., ebsco</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>EBSCONET</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.ebsconet.com</t>
-        </is>
-      </c>
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="D3" s="17" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="C3:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Admin, End user, Reports, Orders, Invoices, Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Online, FTP, Email, Other"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>